<commit_message>
updated jam nut receptacle dimensions
</commit_message>
<xml_diff>
--- a/calculations/D38999_24AXXPX_Dimensions.xlsx
+++ b/calculations/D38999_24AXXPX_Dimensions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lelem\git_repositories\projects\D38999-3MF\calculations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1A69DC-BFEF-41DC-9C86-B124CE56835F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48532EEE-18C6-406B-9B44-BC31204DDE16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{58E9E39D-3151-410B-8DC1-39983DB63DF0}"/>
+    <workbookView xWindow="14790" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{58E9E39D-3151-410B-8DC1-39983DB63DF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="133">
   <si>
     <t>A</t>
   </si>
@@ -411,6 +411,30 @@
   </si>
   <si>
     <t>24AJ</t>
+  </si>
+  <si>
+    <t>detent groove depth</t>
+  </si>
+  <si>
+    <t>0.100R</t>
+  </si>
+  <si>
+    <t>M47x1.0-6g</t>
+  </si>
+  <si>
+    <t>internal jam nut thread major diameter</t>
+  </si>
+  <si>
+    <t>external jam nut thread major diameter</t>
+  </si>
+  <si>
+    <t>internal jam nut thread minor diameter</t>
+  </si>
+  <si>
+    <t>external jam nut thread minor diameter</t>
+  </si>
+  <si>
+    <t>jam nut thread pitch</t>
   </si>
 </sst>
 </file>
@@ -458,11 +482,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -801,15 +826,36 @@
   <dimension ref="A1:AH111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.578125" customWidth="1"/>
+    <col min="1" max="1" width="44.9453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.1015625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.3125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.3125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.89453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.20703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="36.3671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="36.7890625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30.83984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="32.83984375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.05078125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.20703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.62890625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="29" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="28.1015625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="28.62890625" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="36.3671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="36.7890625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="26" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="19.26171875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26">
+    <row r="1" spans="1:28">
       <c r="A1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:26">
+    <row r="2" spans="1:28">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -879,17 +925,23 @@
       <c r="W2" t="s">
         <v>96</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="X2" t="s">
         <v>115</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Y2" t="s">
         <v>53</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="Z2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="3" spans="1:26">
+      <c r="AA2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:28">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -959,22 +1011,28 @@
       <c r="W3">
         <v>1.32</v>
       </c>
-      <c r="X3" s="4">
+      <c r="X3">
         <v>6</v>
       </c>
-      <c r="Y3" s="4">
+      <c r="Y3">
         <v>5</v>
       </c>
-      <c r="Z3" s="4">
+      <c r="Z3">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:26">
+      <c r="AA3">
+        <v>0.4</v>
+      </c>
+      <c r="AB3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:28">
       <c r="A5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:26">
+    <row r="6" spans="1:28">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1038,8 +1096,20 @@
       <c r="U6" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="8" spans="1:26">
+      <c r="V6" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="W6" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="X6" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="Y6" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" spans="1:28">
       <c r="A8" t="s">
         <v>116</v>
       </c>
@@ -1103,8 +1173,20 @@
       <c r="U8" s="1">
         <v>16.382999999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:26">
+      <c r="V8" s="4">
+        <v>15.747</v>
+      </c>
+      <c r="W8" s="4">
+        <v>16.974</v>
+      </c>
+      <c r="X8" s="4">
+        <v>15.557</v>
+      </c>
+      <c r="Y8" s="4">
+        <v>16.794</v>
+      </c>
+    </row>
+    <row r="9" spans="1:28">
       <c r="A9" t="s">
         <v>117</v>
       </c>
@@ -1168,8 +1250,20 @@
       <c r="U9" s="1">
         <v>19.558</v>
       </c>
-    </row>
-    <row r="10" spans="1:26">
+      <c r="V9" s="4">
+        <v>18.747</v>
+      </c>
+      <c r="W9" s="4">
+        <v>19.974</v>
+      </c>
+      <c r="X9" s="4">
+        <v>18.556999999999999</v>
+      </c>
+      <c r="Y9" s="4">
+        <v>19.794</v>
+      </c>
+    </row>
+    <row r="10" spans="1:28">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -1233,8 +1327,20 @@
       <c r="U10" s="1">
         <v>22.733000000000001</v>
       </c>
-    </row>
-    <row r="11" spans="1:26">
+      <c r="V10" s="4">
+        <v>23.747</v>
+      </c>
+      <c r="W10" s="4">
+        <v>24.974</v>
+      </c>
+      <c r="X10" s="4">
+        <v>23.55</v>
+      </c>
+      <c r="Y10" s="4">
+        <v>24.794</v>
+      </c>
+    </row>
+    <row r="11" spans="1:28">
       <c r="A11" t="s">
         <v>119</v>
       </c>
@@ -1298,8 +1404,20 @@
       <c r="U11" s="1">
         <v>25.907999999999998</v>
       </c>
-    </row>
-    <row r="12" spans="1:26">
+      <c r="V11" s="4">
+        <v>26.747</v>
+      </c>
+      <c r="W11" s="4">
+        <v>27.974</v>
+      </c>
+      <c r="X11" s="4">
+        <v>26.55</v>
+      </c>
+      <c r="Y11" s="4">
+        <v>27.794</v>
+      </c>
+    </row>
+    <row r="12" spans="1:28">
       <c r="A12" t="s">
         <v>120</v>
       </c>
@@ -1363,8 +1481,20 @@
       <c r="U12" s="1">
         <v>30.772099999999998</v>
       </c>
-    </row>
-    <row r="13" spans="1:26">
+      <c r="V12" s="4">
+        <v>30.747</v>
+      </c>
+      <c r="W12" s="4">
+        <v>31.974</v>
+      </c>
+      <c r="X12" s="4">
+        <v>30.55</v>
+      </c>
+      <c r="Y12" s="4">
+        <v>31.794</v>
+      </c>
+    </row>
+    <row r="13" spans="1:28">
       <c r="A13" t="s">
         <v>121</v>
       </c>
@@ -1428,8 +1558,20 @@
       <c r="U13" s="1">
         <v>32.3596</v>
       </c>
-    </row>
-    <row r="14" spans="1:26">
+      <c r="V13" s="4">
+        <v>33.747</v>
+      </c>
+      <c r="W13" s="4">
+        <v>34.973999999999997</v>
+      </c>
+      <c r="X13" s="4">
+        <v>33.549999999999997</v>
+      </c>
+      <c r="Y13" s="4">
+        <v>34.793999999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:28">
       <c r="A14" t="s">
         <v>122</v>
       </c>
@@ -1493,8 +1635,20 @@
       <c r="U14" s="1">
         <v>35.534599999999998</v>
       </c>
-    </row>
-    <row r="15" spans="1:26">
+      <c r="V14" s="4">
+        <v>36.747</v>
+      </c>
+      <c r="W14" s="4">
+        <v>37.973999999999997</v>
+      </c>
+      <c r="X14" s="4">
+        <v>36.549999999999997</v>
+      </c>
+      <c r="Y14" s="4">
+        <v>37.793999999999997</v>
+      </c>
+    </row>
+    <row r="15" spans="1:28">
       <c r="A15" t="s">
         <v>123</v>
       </c>
@@ -1558,8 +1712,20 @@
       <c r="U15" s="1">
         <v>38.709600000000002</v>
       </c>
-    </row>
-    <row r="16" spans="1:26">
+      <c r="V15" s="4">
+        <v>39.747</v>
+      </c>
+      <c r="W15" s="4">
+        <v>40.973999999999997</v>
+      </c>
+      <c r="X15" s="4">
+        <v>39.549999999999997</v>
+      </c>
+      <c r="Y15" s="4">
+        <v>40.793999999999997</v>
+      </c>
+    </row>
+    <row r="16" spans="1:28">
       <c r="A16" t="s">
         <v>124</v>
       </c>
@@ -1622,6 +1788,18 @@
       </c>
       <c r="U16" s="1">
         <v>41.884599999999999</v>
+      </c>
+      <c r="V16" s="4">
+        <v>42.747</v>
+      </c>
+      <c r="W16" s="4">
+        <v>43.973999999999997</v>
+      </c>
+      <c r="X16" s="4">
+        <v>42.55</v>
+      </c>
+      <c r="Y16" s="4">
+        <v>43.793999999999997</v>
       </c>
     </row>
     <row r="18" spans="1:34">
@@ -2257,7 +2435,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:12">
+    <row r="65" spans="1:16">
       <c r="A65" t="s">
         <v>1</v>
       </c>
@@ -2271,7 +2449,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:12">
+    <row r="66" spans="1:16">
       <c r="A66" t="s">
         <v>2</v>
       </c>
@@ -2285,7 +2463,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:12">
+    <row r="67" spans="1:16">
       <c r="A67" t="s">
         <v>3</v>
       </c>
@@ -2299,7 +2477,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:12">
+    <row r="68" spans="1:16">
       <c r="A68" t="s">
         <v>4</v>
       </c>
@@ -2313,7 +2491,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:12">
+    <row r="69" spans="1:16">
       <c r="A69" t="s">
         <v>7</v>
       </c>
@@ -2327,7 +2505,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:12">
+    <row r="70" spans="1:16">
       <c r="A70" t="s">
         <v>8</v>
       </c>
@@ -2341,7 +2519,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:12">
+    <row r="71" spans="1:16">
       <c r="A71" t="s">
         <v>9</v>
       </c>
@@ -2355,17 +2533,17 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:12">
+    <row r="73" spans="1:16">
       <c r="A73" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:12">
+    <row r="74" spans="1:16">
       <c r="A74">
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:12">
+    <row r="75" spans="1:16">
       <c r="A75" t="s">
         <v>17</v>
       </c>
@@ -2387,8 +2565,20 @@
       <c r="G75" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="76" spans="1:12">
+      <c r="H75" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I75" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="J75" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="K75" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="76" spans="1:16">
       <c r="A76" t="s">
         <v>0</v>
       </c>
@@ -2410,9 +2600,24 @@
       <c r="G76">
         <v>16.100000000000001</v>
       </c>
-      <c r="L76" s="1"/>
-    </row>
-    <row r="77" spans="1:12">
+      <c r="H76" s="4">
+        <v>15.747</v>
+      </c>
+      <c r="I76" s="4">
+        <v>16.974</v>
+      </c>
+      <c r="J76" s="4">
+        <v>15.557</v>
+      </c>
+      <c r="K76" s="4">
+        <v>16.794</v>
+      </c>
+      <c r="M76" s="4"/>
+      <c r="N76" s="4"/>
+      <c r="O76" s="4"/>
+      <c r="P76" s="4"/>
+    </row>
+    <row r="77" spans="1:16">
       <c r="A77" t="s">
         <v>6</v>
       </c>
@@ -2434,9 +2639,21 @@
       <c r="G77">
         <v>19.100000000000001</v>
       </c>
-      <c r="L77" s="1"/>
-    </row>
-    <row r="78" spans="1:12">
+      <c r="H77" s="4">
+        <v>18.747</v>
+      </c>
+      <c r="I77" s="4">
+        <v>19.974</v>
+      </c>
+      <c r="J77" s="4">
+        <v>18.556999999999999</v>
+      </c>
+      <c r="K77" s="4">
+        <v>19.794</v>
+      </c>
+      <c r="O77" s="1"/>
+    </row>
+    <row r="78" spans="1:16">
       <c r="A78" t="s">
         <v>1</v>
       </c>
@@ -2458,9 +2675,22 @@
       <c r="G78">
         <v>24.1</v>
       </c>
-      <c r="L78" s="1"/>
-    </row>
-    <row r="79" spans="1:12">
+      <c r="H78" s="4">
+        <v>23.747</v>
+      </c>
+      <c r="I78" s="4">
+        <v>24.974</v>
+      </c>
+      <c r="J78" s="4">
+        <v>23.55</v>
+      </c>
+      <c r="K78" s="4">
+        <v>24.794</v>
+      </c>
+      <c r="N78" s="5"/>
+      <c r="O78" s="1"/>
+    </row>
+    <row r="79" spans="1:16">
       <c r="A79" t="s">
         <v>2</v>
       </c>
@@ -2482,9 +2712,22 @@
       <c r="G79">
         <v>27.1</v>
       </c>
-      <c r="L79" s="1"/>
-    </row>
-    <row r="80" spans="1:12">
+      <c r="H79" s="4">
+        <v>26.747</v>
+      </c>
+      <c r="I79" s="4">
+        <v>27.974</v>
+      </c>
+      <c r="J79" s="4">
+        <v>26.55</v>
+      </c>
+      <c r="K79" s="4">
+        <v>27.794</v>
+      </c>
+      <c r="N79" s="5"/>
+      <c r="O79" s="1"/>
+    </row>
+    <row r="80" spans="1:16">
       <c r="A80" t="s">
         <v>3</v>
       </c>
@@ -2506,9 +2749,22 @@
       <c r="G80">
         <v>31.1</v>
       </c>
-      <c r="L80" s="1"/>
-    </row>
-    <row r="81" spans="1:12">
+      <c r="H80" s="4">
+        <v>30.747</v>
+      </c>
+      <c r="I80" s="4">
+        <v>31.974</v>
+      </c>
+      <c r="J80" s="4">
+        <v>30.55</v>
+      </c>
+      <c r="K80" s="4">
+        <v>31.794</v>
+      </c>
+      <c r="N80" s="5"/>
+      <c r="O80" s="1"/>
+    </row>
+    <row r="81" spans="1:16">
       <c r="A81" t="s">
         <v>4</v>
       </c>
@@ -2530,9 +2786,22 @@
       <c r="G81">
         <v>34.1</v>
       </c>
-      <c r="L81" s="1"/>
-    </row>
-    <row r="82" spans="1:12">
+      <c r="H81" s="4">
+        <v>33.747</v>
+      </c>
+      <c r="I81" s="4">
+        <v>34.973999999999997</v>
+      </c>
+      <c r="J81" s="4">
+        <v>33.549999999999997</v>
+      </c>
+      <c r="K81" s="4">
+        <v>34.793999999999997</v>
+      </c>
+      <c r="N81" s="5"/>
+      <c r="O81" s="1"/>
+    </row>
+    <row r="82" spans="1:16">
       <c r="A82" t="s">
         <v>7</v>
       </c>
@@ -2554,9 +2823,21 @@
       <c r="G82">
         <v>37.1</v>
       </c>
-      <c r="L82" s="1"/>
-    </row>
-    <row r="83" spans="1:12">
+      <c r="H82" s="4">
+        <v>36.747</v>
+      </c>
+      <c r="I82" s="4">
+        <v>37.973999999999997</v>
+      </c>
+      <c r="J82" s="4">
+        <v>36.549999999999997</v>
+      </c>
+      <c r="K82" s="4">
+        <v>37.793999999999997</v>
+      </c>
+      <c r="N82" s="5"/>
+    </row>
+    <row r="83" spans="1:16">
       <c r="A83" t="s">
         <v>8</v>
       </c>
@@ -2578,9 +2859,21 @@
       <c r="G83">
         <v>40.1</v>
       </c>
-      <c r="L83" s="1"/>
-    </row>
-    <row r="84" spans="1:12">
+      <c r="H83" s="4">
+        <v>39.747</v>
+      </c>
+      <c r="I83" s="4">
+        <v>40.973999999999997</v>
+      </c>
+      <c r="J83" s="4">
+        <v>39.549999999999997</v>
+      </c>
+      <c r="K83" s="4">
+        <v>40.793999999999997</v>
+      </c>
+      <c r="N83" s="5"/>
+    </row>
+    <row r="84" spans="1:16">
       <c r="A84" t="s">
         <v>9</v>
       </c>
@@ -2602,14 +2895,38 @@
       <c r="G84">
         <v>43.1</v>
       </c>
-      <c r="L84" s="1"/>
-    </row>
-    <row r="87" spans="1:12">
+      <c r="H84" s="4">
+        <v>42.747</v>
+      </c>
+      <c r="I84" s="4">
+        <v>43.973999999999997</v>
+      </c>
+      <c r="J84" s="4">
+        <v>42.55</v>
+      </c>
+      <c r="K84" s="4">
+        <v>43.793999999999997</v>
+      </c>
+      <c r="N84" s="5"/>
+    </row>
+    <row r="85" spans="1:16">
+      <c r="N85" s="5"/>
+    </row>
+    <row r="86" spans="1:16">
+      <c r="N86" s="5"/>
+    </row>
+    <row r="87" spans="1:16">
       <c r="A87" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="89" spans="1:12">
+    <row r="88" spans="1:16">
+      <c r="M88" s="4"/>
+      <c r="N88" s="4"/>
+      <c r="O88" s="4"/>
+      <c r="P88" s="4"/>
+    </row>
+    <row r="89" spans="1:16">
       <c r="A89" t="s">
         <v>17</v>
       </c>
@@ -2620,7 +2937,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="90" spans="1:12">
+    <row r="90" spans="1:16">
       <c r="A90" t="s">
         <v>0</v>
       </c>
@@ -2631,7 +2948,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="91" spans="1:12">
+    <row r="91" spans="1:16">
       <c r="A91" t="s">
         <v>6</v>
       </c>
@@ -2642,7 +2959,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:12">
+    <row r="92" spans="1:16">
       <c r="A92" t="s">
         <v>1</v>
       </c>
@@ -2652,8 +2969,26 @@
       <c r="C92" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="93" spans="1:12">
+      <c r="K92" t="s">
+        <v>127</v>
+      </c>
+      <c r="L92" t="s">
+        <v>126</v>
+      </c>
+      <c r="M92" s="4">
+        <v>46.973999999999997</v>
+      </c>
+      <c r="N92" s="4">
+        <v>46.793999999999997</v>
+      </c>
+      <c r="O92" s="4">
+        <v>45.747</v>
+      </c>
+      <c r="P92" s="4">
+        <v>45.55</v>
+      </c>
+    </row>
+    <row r="93" spans="1:16">
       <c r="A93" t="s">
         <v>2</v>
       </c>
@@ -2664,7 +2999,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:12">
+    <row r="94" spans="1:16">
       <c r="A94" t="s">
         <v>3</v>
       </c>
@@ -2675,7 +3010,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:12">
+    <row r="95" spans="1:16">
       <c r="A95" t="s">
         <v>4</v>
       </c>
@@ -2686,7 +3021,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="96" spans="1:12">
+    <row r="96" spans="1:16">
       <c r="A96" t="s">
         <v>7</v>
       </c>

</xml_diff>